<commit_message>
#31 eSpark and Client BOM added
</commit_message>
<xml_diff>
--- a/Design Files/BLDC-Board-v1.0/BOM/Client BOM BLDC-Board-v1.0.xlsx
+++ b/Design Files/BLDC-Board-v1.0/BOM/Client BOM BLDC-Board-v1.0.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="488" uniqueCount="332">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="488" uniqueCount="331">
   <si>
     <t>#</t>
   </si>
@@ -348,9 +348,6 @@
     <t>TVS DIODE 5V 9.8V SOD923</t>
   </si>
   <si>
-    <t>TVS SURGE PROTECTOR 1-CH 3.3V</t>
-  </si>
-  <si>
     <t>TVS DIODE 28VWM 45.4VC SMB</t>
   </si>
   <si>
@@ -525,9 +522,6 @@
     <t>SOD-923.</t>
   </si>
   <si>
-    <t>SOD-123</t>
-  </si>
-  <si>
     <t>SMB_</t>
   </si>
   <si>
@@ -657,9 +651,6 @@
     <t>ESD9L5.0ST5G</t>
   </si>
   <si>
-    <t>AZ3003-01G</t>
-  </si>
-  <si>
     <t>SMBJ28A-13-F</t>
   </si>
   <si>
@@ -816,9 +807,6 @@
     <t>ON Semiconductor</t>
   </si>
   <si>
-    <t>Amazing</t>
-  </si>
-  <si>
     <t>Diodes</t>
   </si>
   <si>
@@ -1015,6 +1003,15 @@
   </si>
   <si>
     <t>Amphenol</t>
+  </si>
+  <si>
+    <t>20A 350W 16V 4V 3.3V SOD-323 ESD and Surge Protection (TVS/ESD) ROHS</t>
+  </si>
+  <si>
+    <t>SD03</t>
+  </si>
+  <si>
+    <t>MDD</t>
   </si>
 </sst>
 </file>
@@ -1241,9 +1238,6 @@
     <xf numFmtId="0" fontId="5" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1278,6 +1272,9 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1590,9 +1587,9 @@
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
       <c r="H1" s="2"/>
-      <c r="I1" s="14"/>
-      <c r="J1" s="14"/>
-      <c r="K1" s="14"/>
+      <c r="I1" s="27"/>
+      <c r="J1" s="27"/>
+      <c r="K1" s="27"/>
     </row>
     <row r="2" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
@@ -1609,22 +1606,22 @@
         <v>94</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>258</v>
+        <v>255</v>
       </c>
       <c r="I2" s="6" t="s">
-        <v>327</v>
+        <v>323</v>
       </c>
       <c r="J2" s="5" t="s">
-        <v>325</v>
+        <v>321</v>
       </c>
       <c r="K2" s="5" t="s">
-        <v>328</v>
+        <v>324</v>
       </c>
     </row>
     <row r="3" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1643,16 +1640,16 @@
         <v>95</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="H3" s="7" t="s">
-        <v>259</v>
+        <v>256</v>
       </c>
       <c r="I3" s="8" t="s">
-        <v>292</v>
+        <v>288</v>
       </c>
       <c r="J3" s="7">
         <v>4</v>
@@ -1675,54 +1672,54 @@
         <v>96</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="G4" s="10" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="H4" s="9" t="s">
-        <v>259</v>
+        <v>256</v>
       </c>
       <c r="I4" s="10" t="s">
-        <v>293</v>
+        <v>289</v>
       </c>
       <c r="J4" s="9">
         <v>1</v>
       </c>
       <c r="K4" s="9"/>
     </row>
-    <row r="5" spans="1:11" s="24" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="18"/>
-      <c r="B5" s="19">
+    <row r="5" spans="1:11" s="23" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="17"/>
+      <c r="B5" s="18">
         <f>ROW(B5) - ROW($B$2)</f>
         <v>3</v>
       </c>
-      <c r="C5" s="25" t="s">
+      <c r="C5" s="24" t="s">
         <v>2</v>
       </c>
-      <c r="D5" s="26" t="s">
+      <c r="D5" s="25" t="s">
         <v>28</v>
       </c>
-      <c r="E5" s="27" t="s">
+      <c r="E5" s="26" t="s">
         <v>97</v>
       </c>
-      <c r="F5" s="26" t="s">
-        <v>162</v>
-      </c>
-      <c r="G5" s="27" t="s">
-        <v>201</v>
-      </c>
-      <c r="H5" s="26" t="s">
-        <v>259</v>
-      </c>
-      <c r="I5" s="27" t="s">
-        <v>294</v>
-      </c>
-      <c r="J5" s="26">
+      <c r="F5" s="25" t="s">
+        <v>161</v>
+      </c>
+      <c r="G5" s="26" t="s">
+        <v>199</v>
+      </c>
+      <c r="H5" s="25" t="s">
+        <v>256</v>
+      </c>
+      <c r="I5" s="26" t="s">
+        <v>290</v>
+      </c>
+      <c r="J5" s="25">
         <v>2</v>
       </c>
-      <c r="K5" s="23" t="s">
-        <v>330</v>
+      <c r="K5" s="22" t="s">
+        <v>326</v>
       </c>
     </row>
     <row r="6" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1741,16 +1738,16 @@
         <v>98</v>
       </c>
       <c r="F6" s="9" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="G6" s="10" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="H6" s="9" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="I6" s="10" t="s">
-        <v>295</v>
+        <v>291</v>
       </c>
       <c r="J6" s="9">
         <v>2</v>
@@ -1773,16 +1770,16 @@
         <v>99</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="G7" s="8" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="H7" s="7" t="s">
-        <v>259</v>
+        <v>256</v>
       </c>
       <c r="I7" s="8" t="s">
-        <v>296</v>
+        <v>292</v>
       </c>
       <c r="J7" s="7">
         <v>1</v>
@@ -1805,16 +1802,16 @@
         <v>100</v>
       </c>
       <c r="F8" s="9" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="G8" s="10" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="H8" s="9" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
       <c r="I8" s="10" t="s">
-        <v>297</v>
+        <v>293</v>
       </c>
       <c r="J8" s="9">
         <v>6</v>
@@ -1837,16 +1834,16 @@
         <v>101</v>
       </c>
       <c r="F9" s="7" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="G9" s="8" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="H9" s="7" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
       <c r="I9" s="8" t="s">
-        <v>292</v>
+        <v>288</v>
       </c>
       <c r="J9" s="7">
         <v>1</v>
@@ -1869,16 +1866,16 @@
         <v>102</v>
       </c>
       <c r="F10" s="9" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="G10" s="10" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="H10" s="9" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="I10" s="10" t="s">
-        <v>298</v>
+        <v>294</v>
       </c>
       <c r="J10" s="9">
         <v>1</v>
@@ -1901,16 +1898,16 @@
         <v>103</v>
       </c>
       <c r="F11" s="7" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="G11" s="8" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="H11" s="7" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
       <c r="I11" s="8" t="s">
-        <v>299</v>
+        <v>295</v>
       </c>
       <c r="J11" s="7">
         <v>3</v>
@@ -1933,16 +1930,16 @@
         <v>104</v>
       </c>
       <c r="F12" s="9" t="s">
-        <v>326</v>
+        <v>322</v>
       </c>
       <c r="G12" s="10" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="H12" s="9" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="I12" s="10" t="s">
-        <v>300</v>
+        <v>296</v>
       </c>
       <c r="J12" s="9">
         <v>6</v>
@@ -1965,16 +1962,16 @@
         <v>105</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="G13" s="8" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="H13" s="7" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="I13" s="8" t="s">
-        <v>301</v>
+        <v>297</v>
       </c>
       <c r="J13" s="7">
         <v>3</v>
@@ -1997,16 +1994,16 @@
         <v>106</v>
       </c>
       <c r="F14" s="9" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="G14" s="10" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="H14" s="9" t="s">
-        <v>259</v>
+        <v>256</v>
       </c>
       <c r="I14" s="10" t="s">
-        <v>293</v>
+        <v>289</v>
       </c>
       <c r="J14" s="9">
         <v>1</v>
@@ -2029,16 +2026,16 @@
         <v>107</v>
       </c>
       <c r="F15" s="7" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="G15" s="8" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="H15" s="7" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="I15" s="8" t="s">
-        <v>302</v>
+        <v>298</v>
       </c>
       <c r="J15" s="7">
         <v>6</v>
@@ -2061,23 +2058,23 @@
         <v>108</v>
       </c>
       <c r="F16" s="9" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="G16" s="10" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="H16" s="9" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="I16" s="10" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="J16" s="9">
         <v>2</v>
       </c>
       <c r="K16" s="9"/>
     </row>
-    <row r="17" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="1"/>
       <c r="B17" s="11">
         <f>ROW(B17) - ROW($B$2)</f>
@@ -2089,20 +2086,20 @@
       <c r="D17" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="E17" s="8" t="s">
-        <v>109</v>
-      </c>
-      <c r="F17" s="7" t="s">
-        <v>168</v>
-      </c>
-      <c r="G17" s="8" t="s">
-        <v>212</v>
-      </c>
-      <c r="H17" s="7" t="s">
-        <v>265</v>
+      <c r="E17" s="9" t="s">
+        <v>328</v>
+      </c>
+      <c r="F17" s="9" t="s">
+        <v>170</v>
+      </c>
+      <c r="G17" s="9" t="s">
+        <v>329</v>
+      </c>
+      <c r="H17" s="9" t="s">
+        <v>330</v>
       </c>
       <c r="I17" s="10" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="J17" s="7">
         <v>2</v>
@@ -2122,19 +2119,19 @@
         <v>41</v>
       </c>
       <c r="E18" s="10" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="F18" s="9" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="G18" s="10" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="H18" s="9" t="s">
-        <v>266</v>
+        <v>262</v>
       </c>
       <c r="I18" s="10" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="J18" s="9">
         <v>1</v>
@@ -2154,19 +2151,19 @@
         <v>42</v>
       </c>
       <c r="E19" s="8" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="F19" s="7" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="G19" s="8" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="H19" s="7" t="s">
-        <v>267</v>
+        <v>263</v>
       </c>
       <c r="I19" s="10" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="J19" s="7">
         <v>1</v>
@@ -2186,19 +2183,19 @@
         <v>43</v>
       </c>
       <c r="E20" s="10" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="F20" s="9" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="G20" s="10" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="H20" s="9" t="s">
-        <v>268</v>
+        <v>264</v>
       </c>
       <c r="I20" s="10" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="J20" s="9">
         <v>4</v>
@@ -2218,19 +2215,19 @@
         <v>44</v>
       </c>
       <c r="E21" s="8" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="F21" s="7" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="G21" s="8" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="H21" s="7" t="s">
-        <v>266</v>
+        <v>262</v>
       </c>
       <c r="I21" s="10" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="J21" s="7">
         <v>4</v>
@@ -2250,19 +2247,19 @@
         <v>45</v>
       </c>
       <c r="E22" s="10" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="F22" s="9" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="G22" s="10" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="H22" s="9" t="s">
-        <v>269</v>
+        <v>265</v>
       </c>
       <c r="I22" s="10" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="J22" s="9">
         <v>4</v>
@@ -2282,19 +2279,19 @@
         <v>46</v>
       </c>
       <c r="E23" s="8" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="F23" s="7" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="G23" s="8" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="H23" s="7" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="I23" s="10" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="J23" s="7">
         <v>8</v>
@@ -2314,19 +2311,19 @@
         <v>47</v>
       </c>
       <c r="E24" s="10" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="F24" s="9" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="G24" s="10" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="H24" s="9" t="s">
-        <v>270</v>
+        <v>266</v>
       </c>
       <c r="I24" s="10" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="J24" s="9">
         <v>4</v>
@@ -2346,19 +2343,19 @@
         <v>48</v>
       </c>
       <c r="E25" s="8" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="F25" s="9" t="s">
-        <v>326</v>
+        <v>322</v>
       </c>
       <c r="G25" s="8" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="H25" s="7" t="s">
-        <v>271</v>
+        <v>267</v>
       </c>
       <c r="I25" s="10" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="J25" s="7">
         <v>1</v>
@@ -2378,19 +2375,19 @@
         <v>49</v>
       </c>
       <c r="E26" s="10" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="F26" s="9" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="G26" s="10" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
       <c r="H26" s="9" t="s">
-        <v>272</v>
+        <v>268</v>
       </c>
       <c r="I26" s="10" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="J26" s="9">
         <v>2</v>
@@ -2410,19 +2407,19 @@
         <v>50</v>
       </c>
       <c r="E27" s="8" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="F27" s="7" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="G27" s="8" t="s">
-        <v>303</v>
+        <v>299</v>
       </c>
       <c r="H27" s="7" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
       <c r="I27" s="10" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="J27" s="7">
         <v>1</v>
@@ -2442,19 +2439,19 @@
         <v>51</v>
       </c>
       <c r="E28" s="10" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="F28" s="9" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="G28" s="10" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="H28" s="9" t="s">
-        <v>272</v>
+        <v>268</v>
       </c>
       <c r="I28" s="10" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="J28" s="9">
         <v>1</v>
@@ -2474,19 +2471,19 @@
         <v>52</v>
       </c>
       <c r="E29" s="8" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F29" s="9" t="s">
-        <v>326</v>
+        <v>322</v>
       </c>
       <c r="G29" s="8" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="H29" s="7" t="s">
-        <v>273</v>
+        <v>269</v>
       </c>
       <c r="I29" s="10" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="J29" s="7">
         <v>4</v>
@@ -2506,19 +2503,19 @@
         <v>53</v>
       </c>
       <c r="E30" s="10" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="F30" s="9" t="s">
-        <v>326</v>
+        <v>322</v>
       </c>
       <c r="G30" s="10" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="H30" s="9" t="s">
-        <v>273</v>
+        <v>269</v>
       </c>
       <c r="I30" s="10" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="J30" s="9">
         <v>1</v>
@@ -2538,19 +2535,19 @@
         <v>54</v>
       </c>
       <c r="E31" s="8" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="F31" s="9" t="s">
-        <v>326</v>
+        <v>322</v>
       </c>
       <c r="G31" s="8">
         <v>1715721</v>
       </c>
       <c r="H31" s="7" t="s">
-        <v>274</v>
+        <v>270</v>
       </c>
       <c r="I31" s="10" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="J31" s="7">
         <v>3</v>
@@ -2570,19 +2567,19 @@
         <v>55</v>
       </c>
       <c r="E32" s="10" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F32" s="9" t="s">
-        <v>326</v>
+        <v>322</v>
       </c>
       <c r="G32" s="10" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="H32" s="9" t="s">
-        <v>275</v>
+        <v>271</v>
       </c>
       <c r="I32" s="10" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="J32" s="9">
         <v>4</v>
@@ -2602,19 +2599,19 @@
         <v>56</v>
       </c>
       <c r="E33" s="8" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F33" s="7" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="G33" s="8" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="H33" s="7" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="I33" s="10" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="J33" s="7">
         <v>1</v>
@@ -2634,19 +2631,19 @@
         <v>57</v>
       </c>
       <c r="E34" s="10" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="F34" s="9" t="s">
-        <v>326</v>
+        <v>322</v>
       </c>
       <c r="G34" s="10" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="H34" s="9" t="s">
-        <v>276</v>
+        <v>272</v>
       </c>
       <c r="I34" s="10" t="s">
-        <v>304</v>
+        <v>300</v>
       </c>
       <c r="J34" s="9">
         <v>1</v>
@@ -2666,19 +2663,19 @@
         <v>58</v>
       </c>
       <c r="E35" s="8" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F35" s="7" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="G35" s="8" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="H35" s="7" t="s">
-        <v>277</v>
+        <v>273</v>
       </c>
       <c r="I35" s="8" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="J35" s="7">
         <v>3</v>
@@ -2698,19 +2695,19 @@
         <v>59</v>
       </c>
       <c r="E36" s="10" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="F36" s="9" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="G36" s="10" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="H36" s="9" t="s">
-        <v>266</v>
+        <v>262</v>
       </c>
       <c r="I36" s="8" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="J36" s="9">
         <v>4</v>
@@ -2730,19 +2727,19 @@
         <v>60</v>
       </c>
       <c r="E37" s="8" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="F37" s="7" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="G37" s="8" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="H37" s="7" t="s">
-        <v>278</v>
+        <v>274</v>
       </c>
       <c r="I37" s="8" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="J37" s="7">
         <v>4</v>
@@ -2762,19 +2759,19 @@
         <v>61</v>
       </c>
       <c r="E38" s="10" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="F38" s="9" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="G38" s="10" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="H38" s="9" t="s">
-        <v>279</v>
+        <v>275</v>
       </c>
       <c r="I38" s="8" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="J38" s="9">
         <v>4</v>
@@ -2794,19 +2791,19 @@
         <v>62</v>
       </c>
       <c r="E39" s="8" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F39" s="7" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="G39" s="8" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="H39" s="7" t="s">
-        <v>259</v>
+        <v>256</v>
       </c>
       <c r="I39" s="8" t="s">
-        <v>305</v>
+        <v>301</v>
       </c>
       <c r="J39" s="7">
         <v>2</v>
@@ -2826,57 +2823,57 @@
         <v>63</v>
       </c>
       <c r="E40" s="10" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="F40" s="9" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="G40" s="10" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="H40" s="9" t="s">
-        <v>259</v>
+        <v>256</v>
       </c>
       <c r="I40" s="10" t="s">
-        <v>306</v>
+        <v>302</v>
       </c>
       <c r="J40" s="9">
         <v>1</v>
       </c>
       <c r="K40" s="9"/>
     </row>
-    <row r="41" spans="1:11" s="24" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A41" s="18"/>
-      <c r="B41" s="19">
+    <row r="41" spans="1:11" s="23" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A41" s="17"/>
+      <c r="B41" s="18">
         <f>ROW(B41) - ROW($B$2)</f>
         <v>39</v>
       </c>
-      <c r="C41" s="25" t="s">
+      <c r="C41" s="24" t="s">
         <v>19</v>
       </c>
-      <c r="D41" s="26" t="s">
+      <c r="D41" s="25" t="s">
         <v>64</v>
       </c>
-      <c r="E41" s="27" t="s">
-        <v>133</v>
-      </c>
-      <c r="F41" s="26" t="s">
-        <v>185</v>
-      </c>
-      <c r="G41" s="27" t="s">
-        <v>231</v>
-      </c>
-      <c r="H41" s="26" t="s">
-        <v>259</v>
-      </c>
-      <c r="I41" s="27" t="s">
-        <v>294</v>
-      </c>
-      <c r="J41" s="26">
+      <c r="E41" s="26" t="s">
+        <v>132</v>
+      </c>
+      <c r="F41" s="25" t="s">
+        <v>183</v>
+      </c>
+      <c r="G41" s="26" t="s">
+        <v>228</v>
+      </c>
+      <c r="H41" s="25" t="s">
+        <v>256</v>
+      </c>
+      <c r="I41" s="26" t="s">
+        <v>290</v>
+      </c>
+      <c r="J41" s="25">
         <v>2</v>
       </c>
-      <c r="K41" s="23" t="s">
-        <v>330</v>
+      <c r="K41" s="22" t="s">
+        <v>326</v>
       </c>
     </row>
     <row r="42" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -2892,19 +2889,19 @@
         <v>65</v>
       </c>
       <c r="E42" s="10" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="F42" s="9" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="G42" s="10" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="H42" s="9" t="s">
-        <v>259</v>
+        <v>256</v>
       </c>
       <c r="I42" s="10" t="s">
-        <v>307</v>
+        <v>303</v>
       </c>
       <c r="J42" s="9">
         <v>2</v>
@@ -2924,19 +2921,19 @@
         <v>66</v>
       </c>
       <c r="E43" s="8" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F43" s="7" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="G43" s="8" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="H43" s="7" t="s">
-        <v>259</v>
+        <v>256</v>
       </c>
       <c r="I43" s="8" t="s">
-        <v>308</v>
+        <v>304</v>
       </c>
       <c r="J43" s="7">
         <v>14</v>
@@ -2956,19 +2953,19 @@
         <v>67</v>
       </c>
       <c r="E44" s="10" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="F44" s="9" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="G44" s="10" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="H44" s="9" t="s">
-        <v>259</v>
+        <v>256</v>
       </c>
       <c r="I44" s="10" t="s">
-        <v>309</v>
+        <v>305</v>
       </c>
       <c r="J44" s="9">
         <v>1</v>
@@ -2988,19 +2985,19 @@
         <v>68</v>
       </c>
       <c r="E45" s="8" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="F45" s="7" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="G45" s="8" t="s">
-        <v>234</v>
+        <v>231</v>
       </c>
       <c r="H45" s="7" t="s">
-        <v>259</v>
+        <v>256</v>
       </c>
       <c r="I45" s="8" t="s">
-        <v>310</v>
+        <v>306</v>
       </c>
       <c r="J45" s="7">
         <v>1</v>
@@ -3020,19 +3017,19 @@
         <v>69</v>
       </c>
       <c r="E46" s="10" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="F46" s="9" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="G46" s="10" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
       <c r="H46" s="9" t="s">
-        <v>280</v>
+        <v>276</v>
       </c>
       <c r="I46" s="10" t="s">
-        <v>311</v>
+        <v>307</v>
       </c>
       <c r="J46" s="9">
         <v>4</v>
@@ -3052,19 +3049,19 @@
         <v>70</v>
       </c>
       <c r="E47" s="8" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="F47" s="7" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="G47" s="8" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="H47" s="7" t="s">
-        <v>281</v>
+        <v>277</v>
       </c>
       <c r="I47" s="8" t="s">
-        <v>312</v>
+        <v>308</v>
       </c>
       <c r="J47" s="7">
         <v>16</v>
@@ -3084,19 +3081,19 @@
         <v>71</v>
       </c>
       <c r="E48" s="10" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="F48" s="9" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="G48" s="10" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="H48" s="9" t="s">
-        <v>259</v>
+        <v>256</v>
       </c>
       <c r="I48" s="10" t="s">
-        <v>313</v>
+        <v>309</v>
       </c>
       <c r="J48" s="9">
         <v>4</v>
@@ -3116,19 +3113,19 @@
         <v>72</v>
       </c>
       <c r="E49" s="8" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="F49" s="7" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="G49" s="8" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="H49" s="7" t="s">
-        <v>282</v>
+        <v>278</v>
       </c>
       <c r="I49" s="8" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="J49" s="7">
         <v>1</v>
@@ -3148,17 +3145,17 @@
         <v>73</v>
       </c>
       <c r="E50" s="10" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F50" s="9" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="G50" s="10" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="H50" s="9"/>
       <c r="I50" s="10" t="s">
-        <v>315</v>
+        <v>311</v>
       </c>
       <c r="J50" s="9">
         <v>2</v>
@@ -3178,19 +3175,19 @@
         <v>74</v>
       </c>
       <c r="E51" s="8" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="F51" s="7" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="G51" s="8" t="s">
-        <v>240</v>
+        <v>237</v>
       </c>
       <c r="H51" s="7" t="s">
-        <v>259</v>
+        <v>256</v>
       </c>
       <c r="I51" s="8" t="s">
-        <v>316</v>
+        <v>312</v>
       </c>
       <c r="J51" s="7">
         <v>1</v>
@@ -3210,19 +3207,19 @@
         <v>75</v>
       </c>
       <c r="E52" s="10" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="F52" s="9" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="G52" s="10" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="H52" s="9" t="s">
-        <v>259</v>
+        <v>256</v>
       </c>
       <c r="I52" s="10" t="s">
-        <v>317</v>
+        <v>313</v>
       </c>
       <c r="J52" s="9">
         <v>6</v>
@@ -3242,19 +3239,19 @@
         <v>76</v>
       </c>
       <c r="E53" s="8" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="F53" s="7" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="G53" s="8" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
       <c r="H53" s="7" t="s">
-        <v>259</v>
+        <v>256</v>
       </c>
       <c r="I53" s="8" t="s">
-        <v>318</v>
+        <v>314</v>
       </c>
       <c r="J53" s="7">
         <v>4</v>
@@ -3274,19 +3271,19 @@
         <v>77</v>
       </c>
       <c r="E54" s="10" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F54" s="9" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="G54" s="10" t="s">
-        <v>243</v>
+        <v>240</v>
       </c>
       <c r="H54" s="9" t="s">
-        <v>259</v>
+        <v>256</v>
       </c>
       <c r="I54" s="10" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
       <c r="J54" s="9">
         <v>1</v>
@@ -3306,19 +3303,19 @@
         <v>78</v>
       </c>
       <c r="E55" s="8" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="F55" s="7" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="G55" s="8" t="s">
-        <v>244</v>
+        <v>241</v>
       </c>
       <c r="H55" s="7" t="s">
-        <v>283</v>
+        <v>279</v>
       </c>
       <c r="I55" s="8" t="s">
-        <v>320</v>
+        <v>316</v>
       </c>
       <c r="J55" s="7">
         <v>12</v>
@@ -3338,19 +3335,19 @@
         <v>79</v>
       </c>
       <c r="E56" s="10" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="F56" s="9" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="G56" s="10" t="s">
-        <v>245</v>
+        <v>242</v>
       </c>
       <c r="H56" s="9" t="s">
-        <v>259</v>
+        <v>256</v>
       </c>
       <c r="I56" s="10" t="s">
-        <v>321</v>
+        <v>317</v>
       </c>
       <c r="J56" s="9">
         <v>1</v>
@@ -3370,57 +3367,57 @@
         <v>80</v>
       </c>
       <c r="E57" s="8" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="F57" s="7" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="G57" s="8" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="H57" s="7" t="s">
-        <v>259</v>
+        <v>256</v>
       </c>
       <c r="I57" s="8" t="s">
-        <v>322</v>
+        <v>318</v>
       </c>
       <c r="J57" s="7">
         <v>1</v>
       </c>
       <c r="K57" s="7"/>
     </row>
-    <row r="58" spans="1:11" s="24" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A58" s="18"/>
-      <c r="B58" s="19">
+    <row r="58" spans="1:11" s="23" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A58" s="17"/>
+      <c r="B58" s="18">
         <f t="shared" si="0"/>
         <v>56</v>
       </c>
-      <c r="C58" s="20" t="s">
+      <c r="C58" s="19" t="s">
         <v>19</v>
       </c>
-      <c r="D58" s="21" t="s">
+      <c r="D58" s="20" t="s">
         <v>81</v>
       </c>
-      <c r="E58" s="22" t="s">
-        <v>134</v>
-      </c>
-      <c r="F58" s="21" t="s">
-        <v>184</v>
-      </c>
-      <c r="G58" s="22" t="s">
-        <v>232</v>
-      </c>
-      <c r="H58" s="21" t="s">
-        <v>259</v>
-      </c>
-      <c r="I58" s="22" t="s">
-        <v>294</v>
-      </c>
-      <c r="J58" s="21">
+      <c r="E58" s="21" t="s">
+        <v>133</v>
+      </c>
+      <c r="F58" s="20" t="s">
+        <v>182</v>
+      </c>
+      <c r="G58" s="21" t="s">
+        <v>229</v>
+      </c>
+      <c r="H58" s="20" t="s">
+        <v>256</v>
+      </c>
+      <c r="I58" s="21" t="s">
+        <v>290</v>
+      </c>
+      <c r="J58" s="20">
         <v>4</v>
       </c>
-      <c r="K58" s="23" t="s">
-        <v>330</v>
+      <c r="K58" s="22" t="s">
+        <v>326</v>
       </c>
     </row>
     <row r="59" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -3436,19 +3433,19 @@
         <v>82</v>
       </c>
       <c r="E59" s="8" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="F59" s="7" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="G59" s="8" t="s">
-        <v>247</v>
+        <v>244</v>
       </c>
       <c r="H59" s="7" t="s">
-        <v>259</v>
+        <v>256</v>
       </c>
       <c r="I59" s="8" t="s">
-        <v>323</v>
+        <v>319</v>
       </c>
       <c r="J59" s="7">
         <v>1</v>
@@ -3468,19 +3465,19 @@
         <v>83</v>
       </c>
       <c r="E60" s="10" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="F60" s="9" t="s">
-        <v>326</v>
+        <v>322</v>
       </c>
       <c r="G60" s="10" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="H60" s="9" t="s">
-        <v>284</v>
+        <v>280</v>
       </c>
       <c r="I60" s="10" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="J60" s="9">
         <v>1</v>
@@ -3500,19 +3497,19 @@
         <v>84</v>
       </c>
       <c r="E61" s="8" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="F61" s="7" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="G61" s="8" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="H61" s="7" t="s">
-        <v>285</v>
+        <v>281</v>
       </c>
       <c r="I61" s="10" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="J61" s="7">
         <v>1</v>
@@ -3532,19 +3529,19 @@
         <v>85</v>
       </c>
       <c r="E62" s="10" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F62" s="9" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="G62" s="10" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="H62" s="9" t="s">
-        <v>266</v>
+        <v>262</v>
       </c>
       <c r="I62" s="10" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="J62" s="9">
         <v>1</v>
@@ -3564,19 +3561,19 @@
         <v>86</v>
       </c>
       <c r="E63" s="8" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="F63" s="7" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="G63" s="8" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="H63" s="7" t="s">
-        <v>286</v>
+        <v>282</v>
       </c>
       <c r="I63" s="10" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="J63" s="7">
         <v>1</v>
@@ -3596,19 +3593,19 @@
         <v>87</v>
       </c>
       <c r="E64" s="10" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="F64" s="9" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="G64" s="10" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="H64" s="9" t="s">
-        <v>287</v>
+        <v>283</v>
       </c>
       <c r="I64" s="10" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="J64" s="9">
         <v>4</v>
@@ -3628,19 +3625,19 @@
         <v>88</v>
       </c>
       <c r="E65" s="8" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="F65" s="7" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="G65" s="8" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="H65" s="7" t="s">
-        <v>287</v>
+        <v>283</v>
       </c>
       <c r="I65" s="10" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="J65" s="7">
         <v>1</v>
@@ -3660,19 +3657,19 @@
         <v>89</v>
       </c>
       <c r="E66" s="10" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="F66" s="9" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="G66" s="10" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="H66" s="9" t="s">
-        <v>288</v>
+        <v>284</v>
       </c>
       <c r="I66" s="10" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="J66" s="9">
         <v>1</v>
@@ -3692,19 +3689,19 @@
         <v>90</v>
       </c>
       <c r="E67" s="8" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="F67" s="7" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="G67" s="8" t="s">
-        <v>254</v>
+        <v>251</v>
       </c>
       <c r="H67" s="7" t="s">
-        <v>287</v>
+        <v>283</v>
       </c>
       <c r="I67" s="10" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="J67" s="7">
         <v>1</v>
@@ -3724,19 +3721,19 @@
         <v>91</v>
       </c>
       <c r="E68" s="10" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="F68" s="9" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="G68" s="10" t="s">
-        <v>255</v>
+        <v>252</v>
       </c>
       <c r="H68" s="9" t="s">
-        <v>289</v>
+        <v>285</v>
       </c>
       <c r="I68" s="10" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="J68" s="9">
         <v>12</v>
@@ -3752,29 +3749,29 @@
       <c r="C69" s="12" t="s">
         <v>24</v>
       </c>
-      <c r="D69" s="16" t="s">
+      <c r="D69" s="15" t="s">
         <v>92</v>
       </c>
-      <c r="E69" s="17" t="s">
-        <v>159</v>
-      </c>
-      <c r="F69" s="16" t="s">
-        <v>197</v>
-      </c>
-      <c r="G69" s="17" t="s">
-        <v>256</v>
-      </c>
-      <c r="H69" s="16" t="s">
+      <c r="E69" s="16" t="s">
+        <v>158</v>
+      </c>
+      <c r="F69" s="15" t="s">
+        <v>195</v>
+      </c>
+      <c r="G69" s="16" t="s">
+        <v>253</v>
+      </c>
+      <c r="H69" s="15" t="s">
+        <v>286</v>
+      </c>
+      <c r="I69" s="16" t="s">
         <v>290</v>
       </c>
-      <c r="I69" s="17" t="s">
-        <v>294</v>
-      </c>
-      <c r="J69" s="16">
+      <c r="J69" s="15">
         <v>1</v>
       </c>
-      <c r="K69" s="15" t="s">
-        <v>330</v>
+      <c r="K69" s="14" t="s">
+        <v>326</v>
       </c>
     </row>
     <row r="70" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -3790,19 +3787,19 @@
         <v>93</v>
       </c>
       <c r="E70" s="10" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="F70" s="9" t="s">
-        <v>326</v>
+        <v>322</v>
       </c>
       <c r="G70" s="10" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
       <c r="H70" s="9" t="s">
-        <v>291</v>
+        <v>287</v>
       </c>
       <c r="I70" s="10" t="s">
-        <v>324</v>
+        <v>320</v>
       </c>
       <c r="J70" s="9">
         <v>1</v>

</xml_diff>